<commit_message>
fix: add more missing translations
</commit_message>
<xml_diff>
--- a/translations/welsh-translations/december-waste/xlsx/03-select-multiple-prns.xlsx
+++ b/translations/welsh-translations/december-waste/xlsx/03-select-multiple-prns.xlsx
@@ -76,7 +76,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="5" width="24" customWidth="1" hidden="1"/>
@@ -231,8 +231,50 @@
         </is>
       </c>
     </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Prns/SelectMultiplePrns.en.resx::apply_filter</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Prns/SelectMultiplePrns.en.resx</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">apply_filter</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">prns-select-multiple</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/report-data/view-awaiting-acceptance</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Apply filter</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:H7"/>
+  <autoFilter ref="A5:H8"/>
   <mergeCells count="3">
     <mergeCell ref="F1:H1"/>
     <mergeCell ref="F2:H2"/>

</xml_diff>